<commit_message>
fix schedule cell height with absolute positioning; dedupe week goal bars; replace goal dots with dashed rounded tags
</commit_message>
<xml_diff>
--- a/考研复习计划表模板 --地硕.xlsx
+++ b/考研复习计划表模板 --地硕.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="24750" windowHeight="12340"/>
+    <workbookView windowWidth="11950" windowHeight="12350"/>
   </bookViews>
   <sheets>
     <sheet name="月计划模版" sheetId="3" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="66">
   <si>
     <t>月份</t>
   </si>
@@ -112,7 +112,7 @@
     <t>第五周：政治经济学＋新思想概述</t>
   </si>
   <si>
-    <t>第六周：新思想二三、四五、六七、八九、十十一十二、十七</t>
+    <t>第六周：新思想二三四五、六七、八九、十十一十二、十七</t>
   </si>
   <si>
     <t>8月</t>
@@ -1092,7 +1092,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1147,18 +1147,12 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1183,9 +1177,6 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1199,12 +1190,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1576,7 +1561,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr defaultColWidth="8.89090909090909" defaultRowHeight="14" outlineLevelCol="4"/>
   <cols>
     <col min="3" max="3" width="57.7727272727273" customWidth="1"/>
@@ -1605,519 +1590,509 @@
       <c r="A2" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="20"/>
-      <c r="B3" s="21"/>
-      <c r="C3" s="22" t="s">
+      <c r="A3" s="19"/>
+      <c r="B3" s="19"/>
+      <c r="C3" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="20"/>
-      <c r="B4" s="21"/>
-      <c r="C4" s="19" t="s">
+      <c r="A4" s="19"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="18"/>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="20"/>
-      <c r="B5" s="21"/>
-      <c r="C5" s="19" t="s">
+      <c r="A5" s="19"/>
+      <c r="B5" s="19"/>
+      <c r="C5" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="19"/>
-      <c r="E5" s="19"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="18"/>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="20"/>
-      <c r="B6" s="23"/>
-      <c r="C6" s="19" t="s">
+      <c r="A6" s="19"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="19"/>
-      <c r="E6" s="19"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="20"/>
+      <c r="A7" s="19"/>
       <c r="B7" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="24" t="s">
+      <c r="C7" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="25"/>
-      <c r="E7" s="25"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="20"/>
-      <c r="B8" s="20"/>
-      <c r="C8" s="26" t="s">
+      <c r="A8" s="19"/>
+      <c r="B8" s="19"/>
+      <c r="C8" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="25"/>
-      <c r="E8" s="25"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="23"/>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="20"/>
-      <c r="B9" s="20"/>
-      <c r="C9" s="24" t="s">
+      <c r="A9" s="19"/>
+      <c r="B9" s="19"/>
+      <c r="C9" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="25"/>
-      <c r="E9" s="25"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23"/>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="20"/>
-      <c r="B10" s="20"/>
-      <c r="C10" s="24" t="s">
+      <c r="A10" s="19"/>
+      <c r="B10" s="19"/>
+      <c r="C10" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="25"/>
-      <c r="E10" s="25"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="23"/>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="20"/>
-      <c r="B11" s="20"/>
-      <c r="C11" s="24" t="s">
+      <c r="A11" s="19"/>
+      <c r="B11" s="19"/>
+      <c r="C11" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="D11" s="25"/>
-      <c r="E11" s="25"/>
+      <c r="D11" s="23"/>
+      <c r="E11" s="23"/>
     </row>
     <row r="12" ht="42" spans="1:5">
-      <c r="A12" s="20"/>
-      <c r="B12" s="20"/>
-      <c r="C12" s="25" t="s">
+      <c r="A12" s="19"/>
+      <c r="B12" s="19"/>
+      <c r="C12" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="D12" s="27" t="s">
+      <c r="D12" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E12" s="25"/>
+      <c r="E12" s="23"/>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="20"/>
-      <c r="B13" s="20"/>
-      <c r="C13" s="25" t="s">
+      <c r="A13" s="19"/>
+      <c r="B13" s="19"/>
+      <c r="C13" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="D13" s="27"/>
-      <c r="E13" s="25"/>
+      <c r="D13" s="25"/>
+      <c r="E13" s="23"/>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="20"/>
+      <c r="A14" s="19"/>
       <c r="B14" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="28" t="s">
+      <c r="C14" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="D14" s="29"/>
-      <c r="E14" s="29"/>
+      <c r="D14" s="27"/>
+      <c r="E14" s="27"/>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="20"/>
-      <c r="B15" s="20"/>
-      <c r="C15" s="28" t="s">
+      <c r="A15" s="19"/>
+      <c r="B15" s="19"/>
+      <c r="C15" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="D15" s="29"/>
-      <c r="E15" s="29"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="27"/>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="20"/>
-      <c r="B16" s="30"/>
-      <c r="C16" s="28" t="s">
+      <c r="A16" s="19"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="29"/>
-      <c r="E16" s="29"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="27"/>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="20"/>
-      <c r="B17" s="31" t="s">
+      <c r="A17" s="19"/>
+      <c r="B17" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="32" t="s">
+      <c r="C17" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="D17" s="33" t="s">
-        <v>23</v>
-      </c>
-      <c r="E17" s="33" t="s">
+      <c r="D17" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="E17" s="30" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="20"/>
-      <c r="B18" s="34"/>
-      <c r="C18" s="32" t="s">
+      <c r="A18" s="19"/>
+      <c r="B18" s="31"/>
+      <c r="C18" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="D18" s="33" t="s">
-        <v>23</v>
-      </c>
-      <c r="E18" s="33" t="s">
+      <c r="D18" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="E18" s="30" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="30"/>
-      <c r="B19" s="34"/>
-      <c r="C19" s="32" t="s">
+      <c r="A19" s="21"/>
+      <c r="B19" s="31"/>
+      <c r="C19" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="D19" s="33" t="s">
-        <v>23</v>
-      </c>
-      <c r="E19" s="33" t="s">
+      <c r="D19" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="E19" s="30" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="35" t="s">
+      <c r="A20" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="36" t="s">
+      <c r="B20" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="C20" s="19" t="s">
+      <c r="C20" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="D20" s="19"/>
-      <c r="E20" s="19"/>
+      <c r="D20" s="18"/>
+      <c r="E20" s="18"/>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="35"/>
-      <c r="B21" s="37"/>
-      <c r="C21" s="22"/>
-      <c r="D21" s="19"/>
-      <c r="E21" s="19"/>
+      <c r="A21" s="32"/>
+      <c r="B21" s="33" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="D21" s="23"/>
+      <c r="E21" s="23"/>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="35"/>
-      <c r="B22" s="38" t="s">
+      <c r="A22" s="32"/>
+      <c r="B22" s="34"/>
+      <c r="C22" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="D22" s="23"/>
+      <c r="E22" s="23"/>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" s="32"/>
+      <c r="B23" s="34"/>
+      <c r="C23" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="D23" s="23"/>
+      <c r="E23" s="23"/>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" s="32"/>
+      <c r="B24" s="34"/>
+      <c r="C24" s="23" t="s">
+        <v>30</v>
+      </c>
+      <c r="D24" s="25"/>
+      <c r="E24" s="23"/>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" s="32"/>
+      <c r="B25" s="34"/>
+      <c r="C25" s="23" t="s">
+        <v>31</v>
+      </c>
+      <c r="D25" s="25"/>
+      <c r="E25" s="23"/>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" s="32"/>
+      <c r="B26" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="C26" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="D26" s="27"/>
+      <c r="E26" s="27"/>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" s="32"/>
+      <c r="B27" s="34"/>
+      <c r="C27" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="D27" s="27"/>
+      <c r="E27" s="27"/>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" s="32"/>
+      <c r="B28" s="34"/>
+      <c r="C28" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="D28" s="27"/>
+      <c r="E28" s="27"/>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" s="32"/>
+      <c r="B29" s="34"/>
+      <c r="C29" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="D29" s="27"/>
+      <c r="E29" s="27"/>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="A30" s="32"/>
+      <c r="B30" s="35"/>
+      <c r="C30" s="26" t="s">
+        <v>31</v>
+      </c>
+      <c r="D30" s="27"/>
+      <c r="E30" s="27"/>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31" s="32"/>
+      <c r="B31" s="32" t="s">
+        <v>21</v>
+      </c>
+      <c r="C31" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="D31" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="E31" s="30" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="A32" s="36" t="s">
+        <v>37</v>
+      </c>
+      <c r="B32" s="37" t="s">
+        <v>6</v>
+      </c>
+      <c r="C32" s="18"/>
+      <c r="D32" s="18"/>
+      <c r="E32" s="18"/>
+    </row>
+    <row r="33" spans="1:5">
+      <c r="A33" s="36"/>
+      <c r="B33" s="38"/>
+      <c r="C33" s="20"/>
+      <c r="D33" s="18"/>
+      <c r="E33" s="18"/>
+    </row>
+    <row r="34" spans="1:5">
+      <c r="A34" s="36"/>
+      <c r="B34" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="C22" s="24" t="s">
-        <v>27</v>
-      </c>
-      <c r="D22" s="25"/>
-      <c r="E22" s="25"/>
-    </row>
-    <row r="23" spans="1:5">
-      <c r="A23" s="35"/>
-      <c r="B23" s="39"/>
-      <c r="C23" s="26" t="s">
-        <v>28</v>
-      </c>
-      <c r="D23" s="25"/>
-      <c r="E23" s="25"/>
-    </row>
-    <row r="24" spans="1:5">
-      <c r="A24" s="35"/>
-      <c r="B24" s="39"/>
-      <c r="C24" s="24" t="s">
-        <v>29</v>
-      </c>
-      <c r="D24" s="25"/>
-      <c r="E24" s="25"/>
-    </row>
-    <row r="25" ht="42" spans="1:5">
-      <c r="A25" s="35"/>
-      <c r="B25" s="39"/>
-      <c r="C25" s="25" t="s">
-        <v>30</v>
-      </c>
-      <c r="D25" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="E25" s="25"/>
-    </row>
-    <row r="26" spans="1:5">
-      <c r="A26" s="35"/>
-      <c r="B26" s="39"/>
-      <c r="C26" s="25" t="s">
-        <v>31</v>
-      </c>
-      <c r="D26" s="27"/>
-      <c r="E26" s="25"/>
-    </row>
-    <row r="27" spans="1:5">
-      <c r="A27" s="35"/>
-      <c r="B27" s="38" t="s">
+      <c r="C34" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="D34" s="23"/>
+      <c r="E34" s="23"/>
+    </row>
+    <row r="35" spans="1:5">
+      <c r="A35" s="36"/>
+      <c r="B35" s="36"/>
+      <c r="C35" s="24"/>
+      <c r="D35" s="23"/>
+      <c r="E35" s="23"/>
+    </row>
+    <row r="36" spans="1:5">
+      <c r="A36" s="36"/>
+      <c r="B36" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="C27" s="28" t="s">
-        <v>32</v>
-      </c>
-      <c r="D27" s="29"/>
-      <c r="E27" s="29"/>
-    </row>
-    <row r="28" spans="1:5">
-      <c r="A28" s="35"/>
-      <c r="B28" s="39"/>
-      <c r="C28" s="28" t="s">
-        <v>33</v>
-      </c>
-      <c r="D28" s="29"/>
-      <c r="E28" s="29"/>
-    </row>
-    <row r="29" spans="1:5">
-      <c r="A29" s="35"/>
-      <c r="B29" s="39"/>
-      <c r="C29" s="28" t="s">
-        <v>34</v>
-      </c>
-      <c r="D29" s="29"/>
-      <c r="E29" s="29"/>
-    </row>
-    <row r="30" spans="1:5">
-      <c r="A30" s="35"/>
-      <c r="B30" s="39"/>
-      <c r="C30" s="28" t="s">
-        <v>35</v>
-      </c>
-      <c r="D30" s="29"/>
-      <c r="E30" s="29"/>
-    </row>
-    <row r="31" spans="1:5">
-      <c r="A31" s="35"/>
-      <c r="B31" s="40"/>
-      <c r="C31" s="28" t="s">
-        <v>31</v>
-      </c>
-      <c r="D31" s="29"/>
-      <c r="E31" s="29"/>
-    </row>
-    <row r="32" spans="1:5">
-      <c r="A32" s="35"/>
-      <c r="B32" s="35" t="s">
+      <c r="C36" s="26"/>
+      <c r="D36" s="27"/>
+      <c r="E36" s="27"/>
+    </row>
+    <row r="37" spans="1:5">
+      <c r="A37" s="36"/>
+      <c r="B37" s="36" t="s">
         <v>21</v>
       </c>
-      <c r="C32" s="32" t="s">
-        <v>36</v>
-      </c>
-      <c r="D32" s="33" t="s">
-        <v>23</v>
-      </c>
-      <c r="E32" s="33" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5">
-      <c r="A33" s="41" t="s">
-        <v>37</v>
-      </c>
-      <c r="B33" s="42" t="s">
+      <c r="C37" s="29" t="s">
+        <v>23</v>
+      </c>
+      <c r="D37" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="E37" s="30" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5">
+      <c r="A38" s="39" t="s">
+        <v>39</v>
+      </c>
+      <c r="B38" s="40" t="s">
         <v>6</v>
       </c>
-      <c r="C33" s="19"/>
-      <c r="D33" s="19"/>
-      <c r="E33" s="19"/>
-    </row>
-    <row r="34" spans="1:5">
-      <c r="A34" s="41"/>
-      <c r="B34" s="43"/>
-      <c r="C34" s="22"/>
-      <c r="D34" s="19"/>
-      <c r="E34" s="19"/>
-    </row>
-    <row r="35" spans="1:5">
-      <c r="A35" s="41"/>
-      <c r="B35" s="41" t="s">
+      <c r="C38" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="D38" s="18"/>
+      <c r="E38" s="18"/>
+    </row>
+    <row r="39" spans="1:5">
+      <c r="A39" s="39"/>
+      <c r="B39" s="41"/>
+      <c r="C39" s="20"/>
+      <c r="D39" s="18"/>
+      <c r="E39" s="18"/>
+    </row>
+    <row r="40" spans="1:5">
+      <c r="A40" s="39"/>
+      <c r="B40" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="C35" s="24" t="s">
-        <v>38</v>
-      </c>
-      <c r="D35" s="25"/>
-      <c r="E35" s="25"/>
-    </row>
-    <row r="36" spans="1:5">
-      <c r="A36" s="41"/>
-      <c r="B36" s="41"/>
-      <c r="C36" s="26"/>
-      <c r="D36" s="25"/>
-      <c r="E36" s="25"/>
-    </row>
-    <row r="37" spans="1:5">
-      <c r="A37" s="41"/>
-      <c r="B37" s="41" t="s">
+      <c r="C40" s="22"/>
+      <c r="D40" s="23"/>
+      <c r="E40" s="23"/>
+    </row>
+    <row r="41" spans="1:5">
+      <c r="A41" s="39"/>
+      <c r="B41" s="39"/>
+      <c r="C41" s="24"/>
+      <c r="D41" s="23"/>
+      <c r="E41" s="23"/>
+    </row>
+    <row r="42" spans="1:5">
+      <c r="A42" s="39"/>
+      <c r="B42" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="C37" s="28"/>
-      <c r="D37" s="29"/>
-      <c r="E37" s="29"/>
-    </row>
-    <row r="38" spans="1:5">
-      <c r="A38" s="41"/>
-      <c r="B38" s="41" t="s">
+      <c r="C42" s="26"/>
+      <c r="D42" s="26"/>
+      <c r="E42" s="26"/>
+    </row>
+    <row r="43" spans="1:5">
+      <c r="A43" s="39"/>
+      <c r="B43" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="C38" s="32" t="s">
-        <v>23</v>
-      </c>
-      <c r="D38" s="33" t="s">
-        <v>23</v>
-      </c>
-      <c r="E38" s="33" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5">
-      <c r="A39" s="44" t="s">
+      <c r="C43" s="29" t="s">
+        <v>23</v>
+      </c>
+      <c r="D43" s="29" t="s">
+        <v>23</v>
+      </c>
+      <c r="E43" s="29" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5">
+      <c r="A44" s="42" t="s">
         <v>39</v>
       </c>
-      <c r="B39" s="45" t="s">
+      <c r="B44" s="43" t="s">
         <v>6</v>
       </c>
-      <c r="C39" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="D39" s="19"/>
-      <c r="E39" s="19"/>
-    </row>
-    <row r="40" spans="1:5">
-      <c r="A40" s="44"/>
-      <c r="B40" s="46"/>
-      <c r="C40" s="22"/>
-      <c r="D40" s="19"/>
-      <c r="E40" s="19"/>
-    </row>
-    <row r="41" spans="1:5">
-      <c r="A41" s="44"/>
-      <c r="B41" s="44" t="s">
+      <c r="C44" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="D44" s="18"/>
+      <c r="E44" s="18"/>
+    </row>
+    <row r="45" spans="1:5">
+      <c r="A45" s="42"/>
+      <c r="B45" s="44"/>
+      <c r="C45" s="20"/>
+      <c r="D45" s="18"/>
+      <c r="E45" s="18"/>
+    </row>
+    <row r="46" spans="1:5">
+      <c r="A46" s="42"/>
+      <c r="B46" s="42" t="s">
         <v>12</v>
       </c>
-      <c r="C41" s="24"/>
-      <c r="D41" s="25"/>
-      <c r="E41" s="25"/>
-    </row>
-    <row r="42" spans="1:5">
-      <c r="A42" s="44"/>
-      <c r="B42" s="44"/>
-      <c r="C42" s="26"/>
-      <c r="D42" s="25"/>
-      <c r="E42" s="25"/>
-    </row>
-    <row r="43" spans="1:5">
-      <c r="A43" s="44"/>
-      <c r="B43" s="44" t="s">
-        <v>17</v>
-      </c>
-      <c r="C43" s="28"/>
-      <c r="D43" s="28"/>
-      <c r="E43" s="28"/>
-    </row>
-    <row r="44" spans="1:5">
-      <c r="A44" s="44"/>
-      <c r="B44" s="44" t="s">
-        <v>21</v>
-      </c>
-      <c r="C44" s="32" t="s">
-        <v>23</v>
-      </c>
-      <c r="D44" s="32" t="s">
-        <v>23</v>
-      </c>
-      <c r="E44" s="32" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5">
-      <c r="A45" s="47" t="s">
-        <v>39</v>
-      </c>
-      <c r="B45" s="48" t="s">
-        <v>6</v>
-      </c>
-      <c r="C45" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="D45" s="19"/>
-      <c r="E45" s="19"/>
-    </row>
-    <row r="46" spans="1:5">
-      <c r="A46" s="47"/>
-      <c r="B46" s="49"/>
       <c r="C46" s="22"/>
-      <c r="D46" s="19"/>
-      <c r="E46" s="19"/>
+      <c r="D46" s="22"/>
+      <c r="E46" s="22"/>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="47"/>
-      <c r="B47" s="47" t="s">
-        <v>12</v>
-      </c>
+      <c r="A47" s="42"/>
+      <c r="B47" s="42"/>
       <c r="C47" s="24"/>
       <c r="D47" s="24"/>
       <c r="E47" s="24"/>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="47"/>
-      <c r="B48" s="47"/>
+      <c r="A48" s="42"/>
+      <c r="B48" s="42" t="s">
+        <v>17</v>
+      </c>
       <c r="C48" s="26"/>
       <c r="D48" s="26"/>
       <c r="E48" s="26"/>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="47"/>
-      <c r="B49" s="47" t="s">
-        <v>17</v>
-      </c>
-      <c r="C49" s="28"/>
-      <c r="D49" s="28"/>
-      <c r="E49" s="28"/>
-    </row>
-    <row r="50" spans="1:5">
-      <c r="A50" s="47"/>
-      <c r="B50" s="47" t="s">
+      <c r="A49" s="42"/>
+      <c r="B49" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="C50" s="32" t="s">
-        <v>23</v>
-      </c>
-      <c r="D50" s="32" t="s">
-        <v>23</v>
-      </c>
-      <c r="E50" s="32" t="s">
+      <c r="C49" s="29" t="s">
+        <v>23</v>
+      </c>
+      <c r="D49" s="29" t="s">
+        <v>23</v>
+      </c>
+      <c r="E49" s="29" t="s">
         <v>23</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="17">
     <mergeCell ref="A2:A19"/>
-    <mergeCell ref="A20:A32"/>
-    <mergeCell ref="A33:A38"/>
-    <mergeCell ref="A39:A44"/>
-    <mergeCell ref="A45:A50"/>
+    <mergeCell ref="A20:A31"/>
+    <mergeCell ref="A32:A37"/>
+    <mergeCell ref="A38:A43"/>
+    <mergeCell ref="A44:A49"/>
     <mergeCell ref="B2:B6"/>
     <mergeCell ref="B7:B13"/>
     <mergeCell ref="B14:B16"/>
     <mergeCell ref="B17:B19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="B22:B26"/>
-    <mergeCell ref="B27:B31"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="B39:B40"/>
-    <mergeCell ref="B41:B42"/>
-    <mergeCell ref="B45:B46"/>
-    <mergeCell ref="B47:B48"/>
+    <mergeCell ref="B21:B25"/>
+    <mergeCell ref="B26:B30"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="B44:B45"/>
+    <mergeCell ref="B46:B47"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C3" location="'3月第一周'!A1" display="第一周："/>

</xml_diff>